<commit_message>
Actualizacion automatica 2026-10-22 19:16:18 -0500
</commit_message>
<xml_diff>
--- a/Avances/Estación Meteorológica/Materiales/Inventario Circuito Proyecto de Grado.xlsx
+++ b/Avances/Estación Meteorológica/Materiales/Inventario Circuito Proyecto de Grado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Downloads\Proyecto de grado\Avances\Estación Meteorológica\Materiales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608D11A0-D20C-400A-825F-3EA966FBD65A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA1A835-DFAB-4C17-833D-4CEE659DA76D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="38">
   <si>
     <t>Cantidad total</t>
   </si>
@@ -106,6 +106,39 @@
   </si>
   <si>
     <t>Electroválvula latching 12 V</t>
+  </si>
+  <si>
+    <t>Macho-Hembra</t>
+  </si>
+  <si>
+    <t>1 juego</t>
+  </si>
+  <si>
+    <t>1(Opcional)</t>
+  </si>
+  <si>
+    <t>Hidráulico</t>
+  </si>
+  <si>
+    <t>1(Si no se consigue el CN3065)</t>
+  </si>
+  <si>
+    <t>Electroválvula latching 12 V | N/C</t>
+  </si>
+  <si>
+    <t>Convertidor regulador V (boost)</t>
+  </si>
+  <si>
+    <t>LISTA DE MATERIALES REQUERIDOS</t>
+  </si>
+  <si>
+    <t>Miscelanea</t>
+  </si>
+  <si>
+    <t>Estaño</t>
+  </si>
+  <si>
+    <t>1,25m</t>
   </si>
 </sst>
 </file>
@@ -230,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -268,6 +301,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -548,16 +582,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:D26"/>
+  <dimension ref="B1:I28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="43.5703125" customWidth="1"/>
     <col min="3" max="3" width="10.28515625" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" customWidth="1"/>
+    <col min="7" max="7" width="28.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:4" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="2:9" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="13">
+        <v>46307</v>
+      </c>
+      <c r="G3" s="13">
+        <v>46317</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>20</v>
       </c>
@@ -567,8 +617,17 @@
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="2:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>1</v>
       </c>
@@ -578,8 +637,17 @@
       <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="2:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
@@ -589,8 +657,17 @@
       <c r="D6" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="2:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>3</v>
       </c>
@@ -600,8 +677,15 @@
       <c r="D7" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="2:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G7" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="8"/>
+    </row>
+    <row r="8" spans="2:9" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
@@ -611,62 +695,113 @@
       <c r="D8" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="2:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G8" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I8" s="8"/>
+    </row>
+    <row r="9" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="4">
         <v>1</v>
       </c>
-      <c r="D9" s="8"/>
-    </row>
-    <row r="10" spans="2:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="6">
         <v>2</v>
       </c>
-      <c r="D10" s="7"/>
-    </row>
-    <row r="11" spans="2:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D10" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" s="10">
+        <v>1</v>
+      </c>
+      <c r="I10" s="8"/>
+    </row>
+    <row r="11" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="6">
         <v>3</v>
       </c>
-      <c r="D11" s="7"/>
-    </row>
-    <row r="12" spans="2:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D11" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="4">
         <v>1</v>
       </c>
-      <c r="D12" s="8"/>
-    </row>
-    <row r="13" spans="2:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D12" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="I12" s="8"/>
+    </row>
+    <row r="13" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="4">
         <v>1</v>
       </c>
-      <c r="D13" s="8"/>
-    </row>
-    <row r="14" spans="2:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D13" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C14" s="6">
         <v>2</v>
       </c>
-      <c r="D14" s="8"/>
-    </row>
-    <row r="15" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D14" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
         <v>13</v>
       </c>
@@ -677,7 +812,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:9" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
         <v>14</v>
       </c>
@@ -688,7 +823,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>21</v>
       </c>
@@ -699,72 +834,86 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="10">
         <v>1</v>
       </c>
-      <c r="D18" s="8"/>
-    </row>
-    <row r="19" spans="2:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D18" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="4">
         <v>1</v>
       </c>
-      <c r="D19" s="8"/>
-    </row>
-    <row r="20" spans="2:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D19" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="11" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="4">
         <v>1</v>
       </c>
-      <c r="D20" s="8"/>
-    </row>
-    <row r="21" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D20" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C21" s="10">
         <v>1</v>
       </c>
-      <c r="D21" s="8"/>
-    </row>
-    <row r="22" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D21" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="11" t="s">
         <v>23</v>
       </c>
       <c r="C22" s="4">
         <v>1</v>
       </c>
-      <c r="D22" s="8"/>
-    </row>
-    <row r="23" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D22" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C23" s="6">
         <v>1</v>
       </c>
-      <c r="D23" s="8"/>
-    </row>
-    <row r="24" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D23" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="11" t="s">
         <v>25</v>
       </c>
       <c r="C24" s="6">
         <v>2</v>
       </c>
-      <c r="D24" s="8"/>
-    </row>
-    <row r="25" spans="2:4" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D24" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>0</v>
@@ -773,14 +922,38 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:4" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="9" t="s">
         <v>26</v>
       </c>
       <c r="C26" s="10">
         <v>1</v>
       </c>
-      <c r="D26" s="8"/>
+      <c r="D26" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>